<commit_message>
data(pautas_barrios.json): carga del 23/10, 8.085 entradas, y Filas_no_procesadas_pauta_capital.xlsx — fuente: Pauta RRSS_GLOBAL.xlsx (23/10 15:26)
Crudo: Contexto/Pauta RRSS_GLOBAL.xlsx, sha256 3eebe141f35a6ea8131491aefb9ad6fb8621ab741295cd6e89932b8775b84744
Filas: 4.941 renglones, 0 vacías, 4.941 reales (antes 4.104); entran 1.123 (antes 999),
fuera de Capital 3.776, pendientes 8, duplicadas 34 (12 genuinas, 4 sin métricas,
18 a confirmar por el área).
Piezas (campaña + título): 1.415 (antes 1.325): 90 nuevas, 0 bajas.
Entradas: 8.085 (antes 7.259): barrios 4.289 en 184 barrios, circuitos_sin_barrio 3.341,
toda_capital 455.
Estado: Finalizada 7.067, Vigente 776, Observada 242 (S/D: 0 entradas; el ESTADO viene
recalculado).
Al 23/10: tarjeta "Pauta activa" 210 (86 generales + 124 específicas), antes 121;
108 de 119 circuitos y 31 barrios cubiertos, antes 64 y 0.
Mismas reglas que 55bb3e0. Tamaño: 14.225.443 B -> 15.455.262 B.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Filas_no_procesadas_pauta_capital.xlsx
+++ b/public/data/Filas_no_procesadas_pauta_capital.xlsx
@@ -463,7 +463,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4336</v>
+        <v>4941</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>232</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4104</v>
+        <v>4941</v>
       </c>
     </row>
     <row r="5">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>999</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3065</v>
+        <v>3776</v>
       </c>
     </row>
     <row r="7">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7299</v>
+        <v>8130</v>
       </c>
     </row>
     <row r="13">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7259</v>
+        <v>8085</v>
       </c>
     </row>
     <row r="16">
@@ -649,21 +649,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>La localidad es otra (no es Córdoba Capital)</t>
+          <t>TODAS LAS LOCALIDADES de otro departamento de Córdoba</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1640</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES de otro departamento de Córdoba</t>
+          <t>La localidad es otra (no es Córdoba Capital)</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1413</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="24">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25">
@@ -1200,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2106,7 +2106,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Sin métricas (7 filas): Coincide con otra fila en la clave de duplicado y ninguna de las dos tiene métricas cargadas.</t>
+          <t>Sin métricas (4 filas): Coincide con otra fila en la clave de duplicado y ninguna de las dos tiene métricas cargadas.</t>
         </is>
       </c>
       <c r="B15" s="2" t="n"/>
@@ -2372,80 +2372,42 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>4016</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>PLAN DE REPARACIÓN VIAL INTEGRAL</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Plan de Reparación Vial Integral: Calle Impira</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>010D - CONGRESO, CÓRDOBA CAPITAL, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>A confirmar por el área (18 filas): Coincide con otra fila en la clave de duplicado pero las métricas son distintas: puede ser la misma pieza cargada dos veces o dos piezas distintas.</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>(vacío)</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Sin métricas</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>4015</t>
-        </is>
-      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="n"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Coincide con la fila 4015 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, y ninguna de las dos tiene métricas cargadas. El tablero muestra solo la fila 4015.</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>PLAN DE REPARACIÓN VIAL INTEGRAL-Plan de Reparación Vial Integral: Calle Impira-OBRAS-DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA-010D - CONGRESO, CÓRDOBA CAPITAL, ARGENTINA-Reel</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>4052</v>
+        <v>1056</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>CÓRDOBA PRODUCTIVA</t>
+          <t>HACER PARA CRECER</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Visita a CNH Industrial</t>
+          <t>Hacer para crecer Mejoras en la plaza de barrio Parque Latino (Video)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>010I - PARQUE HORIZONTE, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2455,26 +2417,30 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Público afín agricolaganadero, industria, producción</t>
+          <t>Córdoba Capital de 30 a 60 años sin km agregados ni Advantage +</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>(vacío)</t>
+          <t>INACTIVO</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Sin métricas</t>
+          <t>A confirmar por el área</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>4048</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n"/>
-      <c r="K21" s="4" t="n"/>
+          <t>1055</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>297402</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>1029633</v>
+      </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
@@ -2482,32 +2448,32 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 4048 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, y ninguna de las dos tiene métricas cargadas. El tablero muestra solo la fila 4048.</t>
+          <t>Coincide con la fila 1055 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (297.402 contra 1.029.633). El tablero conserva la fila 1055 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link). En las dos filas el LINK MATERIAL y el TIPO DE MATERIAL están vacíos.</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>CÓRDOBA PRODUCTIVA-Visita a CNH Industrial-PRODUCCIÓN-PROVINCIA DE CÓRDOBA, ARGENTINA-TODAS LAS LOCALIDADES-Reel</t>
+          <t>A05710</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>4053</v>
+        <v>1059</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>CÓRDOBA PRODUCTIVA</t>
+          <t>HACER PARA CRECER</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Visita a CNH Industrial</t>
+          <t>Hacer para crecer Nueva sede de la Universidad Provincial de Córdoba en zona sur (Video)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>010L - VILLA EL LIBERTADOR, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2517,26 +2483,30 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Público afín agricolaganadero, industria, producción</t>
+          <t>Córdoba Capital de 30 a 60 años sin km agregados ni Advantage +</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>(vacío)</t>
+          <t>INACTIVO</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Sin métricas</t>
+          <t>A confirmar por el área</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>4049</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
+          <t>1058</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>846262</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>1084459</v>
+      </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
@@ -2544,62 +2514,108 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 4049 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, y ninguna de las dos tiene métricas cargadas. El tablero muestra solo la fila 4049.</t>
+          <t>Coincide con la fila 1058 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (846.262 contra 1.084.459). El tablero conserva la fila 1058 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link). En las dos filas el LINK MATERIAL y el TIPO DE MATERIAL están vacíos.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>CÓRDOBA PRODUCTIVA-Visita a CNH Industrial-PRODUCCIÓN-PROVINCIA DE CÓRDOBA, ARGENTINA-TODAS LAS LOCALIDADES-Reel</t>
+          <t>A05713</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>A confirmar por el área (13 filas): Coincide con otra fila en la clave de duplicado pero las métricas son distintas: puede ser la misma pieza cargada dos veces o dos piezas distintas.</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
+      <c r="A23" s="2" t="n">
+        <v>1515</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>COMUNICACIÓN INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Visita al Club Rosedal</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>010H - PARQUE CAPITAL, CÓRDOBA CAPITAL, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Barrio Rosedal de 30 a 60 años sin advantage</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>INACTIVO</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar por el área</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>1514</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>105340</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>342430</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Coincide con la fila 1514 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (105.340 contra 342.430). El tablero conserva la fila 1514 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>A06269</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>1056</v>
+        <v>2087</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HACER PARA CRECER</t>
+          <t>COMUNICACIÓN INSTITUCIONAL</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hacer para crecer Mejoras en la plaza de barrio Parque Latino (Video)</t>
+          <t>Nos vemos en la Plaza Prussia</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>010I - PARQUE HORIZONTE, CÓRDOBA CAPITAL, ARGENTINA</t>
+          <t>011G - PARQUE REPUBLICA, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Córdoba Capital de 30 a 60 años sin km agregados ni Advantage +</t>
+          <t>Barrio Industrial Oeste de 30 a 60 años sin km agregados</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2614,14 +2630,14 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>1055</t>
+          <t>2086</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>297402</v>
+        <v>24950</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>1029633</v>
+        <v>10169</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
@@ -2630,32 +2646,32 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 1055 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (297.402 contra 1.029.633). El tablero conserva la fila 1055 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link). En las dos filas el LINK MATERIAL y el TIPO DE MATERIAL están vacíos.</t>
+          <t>Coincide con la fila 2086 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (24.950 contra 10.169). El tablero conserva la fila 2086 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>A05710</t>
+          <t>A06300</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>1059</v>
+        <v>2819</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>HACER PARA CRECER</t>
+          <t>EMPLEO +26</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Hacer para crecer Nueva sede de la Universidad Provincial de Córdoba en zona sur (Video)</t>
+          <t>Pieza 1: Formá parte</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>010L - VILLA EL LIBERTADOR, CÓRDOBA CAPITAL, ARGENTINA</t>
+          <t>TODAS LAS LOCALIDADES</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2665,12 +2681,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Córdoba Capital de 30 a 60 años sin km agregados ni Advantage +</t>
+          <t>Hombres y mujeres desde 26 a 60 años</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>INACTIVO</t>
+          <t>OBSERVADO</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2680,63 +2696,63 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>1058</t>
+          <t>2805</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>846262</v>
+        <v>647892</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>1084459</v>
+        <v>616641</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+          <t>Tiene ESTADO = ACTIVO</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 1058 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (846.262 contra 1.084.459). El tablero conserva la fila 1058 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link). En las dos filas el LINK MATERIAL y el TIPO DE MATERIAL están vacíos.</t>
+          <t>Coincide con la fila 2805 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (647.892 contra 616.641). El tablero conserva la fila 2805 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>A05713</t>
+          <t>A07623</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>1515</v>
+        <v>2820</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
+          <t>EMPLEO +26</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Visita al Club Rosedal</t>
+          <t>Pieza 2: Carrusel General</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>010H - PARQUE CAPITAL, CÓRDOBA CAPITAL, ARGENTINA</t>
+          <t>TODAS LAS LOCALIDADES</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Barrio Rosedal de 30 a 60 años sin advantage</t>
+          <t>Hombres y mujeres desde 26 a 60 años</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>INACTIVO</t>
+          <t>OBSERVADO</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2746,63 +2762,63 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>1514</t>
+          <t>2806</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>105340</v>
+        <v>110459</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>342430</v>
+        <v>303096</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+          <t>Tiene ESTADO = ACTIVO</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 1514 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (105.340 contra 342.430). El tablero conserva la fila 1514 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2806 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (110.459 contra 303.096). El tablero conserva la fila 2806 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>A06269</t>
+          <t>A07624</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>2087</v>
+        <v>2821</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
+          <t>EMPLEO +26</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Nos vemos en la Plaza Prussia</t>
+          <t>Pieza 3: Postulantes</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>011G - PARQUE REPUBLICA, CÓRDOBA CAPITAL, ARGENTINA</t>
+          <t>TODAS LAS LOCALIDADES</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Barrio Industrial Oeste de 30 a 60 años sin km agregados</t>
+          <t>Hombres y mujeres desde 26 a 60 años</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>INACTIVO</t>
+          <t>OBSERVADO</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2812,34 +2828,34 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>2086</t>
+          <t>2807</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>24950</v>
+        <v>161979</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>10169</v>
+        <v>144988</v>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+          <t>Tiene ESTADO = ACTIVO</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2086 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (24.950 contra 10.169). El tablero conserva la fila 2086 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2807 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (161.979 contra 144.988). El tablero conserva la fila 2807 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>A06300</t>
+          <t>A07625</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>2819</v>
+        <v>2822</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -2848,7 +2864,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pieza 1: Formá parte</t>
+          <t>Pieza 4: Empresas</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2863,7 +2879,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
+          <t>Intereses B2B | Empresas</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2878,14 +2894,14 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2805</t>
+          <t>2808</t>
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>647892</v>
+        <v>279463</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>349952</v>
+        <v>401761</v>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -2894,18 +2910,18 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2805 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (647.892 contra 349.952). El tablero conserva la fila 2805 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2808 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (279.463 contra 401.761). El tablero conserva la fila 2808 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>A07623</t>
+          <t>A07626</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>2820</v>
+        <v>2823</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -2914,7 +2930,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pieza 2: Carrusel General</t>
+          <t>Pieza 5: Ya está en marcha Empleo +26</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2944,14 +2960,14 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>2806</t>
+          <t>2809</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>110459</v>
+        <v>54884</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>203040</v>
+        <v>279284</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -2960,18 +2976,18 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2806 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (110.459 contra 203.040). El tablero conserva la fila 2806 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2809 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (54.884 contra 279.284). El tablero conserva la fila 2809 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>A07624</t>
+          <t>A07627</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>2821</v>
+        <v>2828</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -2980,7 +2996,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Pieza 3: Postulantes</t>
+          <t>Pieza 7: Otras experiencias Empleo +26</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -3010,14 +3026,14 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>2807</t>
+          <t>2814</t>
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>161979</v>
+        <v>12815</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>72957</v>
+        <v>736704</v>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
@@ -3026,18 +3042,18 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2807 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (161.979 contra 72.957). El tablero conserva la fila 2807 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2814 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (12.815 contra 736.704). El tablero conserva la fila 2814 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>A07625</t>
+          <t>A07632</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>2822</v>
+        <v>2832</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -3046,7 +3062,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Pieza 4: Empresas</t>
+          <t>Pieza 1: Formá parte</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -3061,7 +3077,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Intereses B2B | Empresas</t>
+          <t>Hombres y mujeres desde 26 a 60 años</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -3076,14 +3092,14 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>2808</t>
+          <t>2818</t>
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>279463</v>
+        <v>0</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>243618</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
@@ -3092,47 +3108,43 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2808 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (279.463 contra 243.618). El tablero conserva la fila 2808 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 2818 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las métricas son distintas (impresiones 0 en las dos; inversión 206.843 contra 93.333). El tablero conserva la fila 2818 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>A07626</t>
+          <t>A07636</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>2823</v>
+        <v>3705</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>EMPLEO +26</t>
+          <t>OBRAS QUE TRANSFORMAN</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Pieza 5: Ya está en marcha Empleo +26</t>
+          <t>OBRA-0003 - Avenida Boderau</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>014Q - VILLA WARCALDE, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
-        </is>
-      </c>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>OBSERVADO</t>
+          <t>ACTIVO</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3142,63 +3154,59 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>2809</t>
+          <t>3704</t>
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>54884</v>
+        <v>11995</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>154288</v>
+        <v>13917</v>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Tiene ESTADO = ACTIVO</t>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2809 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (54.884 contra 154.288). El tablero conserva la fila 2809 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 3704 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (11.995 contra 13.917). El tablero conserva la fila 3704 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>A07627</t>
+          <t>A07965</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>2828</v>
+        <v>3706</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>EMPLEO +26</t>
+          <t>OBRAS QUE TRANSFORMAN</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Pieza 7: Otras experiencias Empleo +26</t>
+          <t>OBRA-0003 - Avenida Boderau</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>014P - VILLA RIVERA INDARTE, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
-        </is>
-      </c>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>OBSERVADO</t>
+          <t>ACTIVO</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -3208,63 +3216,59 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>2814</t>
+          <t>3704</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>12815</v>
+        <v>13885</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>452016</v>
+        <v>13917</v>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Tiene ESTADO = ACTIVO</t>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2814 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (12.815 contra 452.016). El tablero conserva la fila 2814 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 3704 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (13.885 contra 13.917). El tablero conserva la fila 3704 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>A07632</t>
+          <t>A07966</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>2830</v>
+        <v>3707</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>EMPLEO +26</t>
+          <t>OBRAS QUE TRANSFORMAN</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Pieza 6: Experiencia Empleo +26 - Inclusión Laboral</t>
+          <t>OBRA-0003 - Avenida Boderau</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>014O - VILLA 9 DE JULIO, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
-        </is>
-      </c>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>OBSERVADO</t>
+          <t>ACTIVO</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3274,63 +3278,59 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>2816</t>
+          <t>3704</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>14846</v>
+        <v>12758</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>5045</v>
+        <v>13917</v>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Tiene ESTADO = ACTIVO</t>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2816 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (14.846 contra 5.045). El tablero conserva la fila 2816 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 3704 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (12.758 contra 13.917). El tablero conserva la fila 3704 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>A07634</t>
+          <t>A07967</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>2831</v>
+        <v>3708</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>EMPLEO +26</t>
+          <t>OBRAS QUE TRANSFORMAN</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Pieza 7: Otras experiencias Empleo +26</t>
+          <t>OBRA-0003 - Avenida Boderau</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>TODAS LAS LOCALIDADES</t>
+          <t>014K - VILLA ALLENDE PARQUE, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
-        </is>
-      </c>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>OBSERVADO</t>
+          <t>ACTIVO</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3340,96 +3340,212 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>2817</t>
+          <t>3704</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>5290</v>
+        <v>13433</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>8408</v>
+        <v>13917</v>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Tiene ESTADO = ACTIVO</t>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Coincide con la fila 2817 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (5.290 contra 8.408). El tablero conserva la fila 2817 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+          <t>Coincide con la fila 3704 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (13.433 contra 13.917). El tablero conserva la fila 3704 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>A07635</t>
+          <t>A07968</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>2832</v>
+        <v>3709</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>EMPLEO +26</t>
+          <t>OBRAS QUE TRANSFORMAN</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Pieza 1: Formá parte</t>
+          <t>OBRA-0003 - Avenida Boderau</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>014C - ARGUELLO SEGUNDO, CÓRDOBA CAPITAL, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar por el área</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>3704</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>15762</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>13917</v>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Coincide con la fila 3704 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (15.762 contra 13.917). El tablero conserva la fila 3704 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>A07969</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>4849</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>PLAN DE REPARACIÓN VIAL INTEGRAL</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Plan de Reparación Vial Integral: Calle Impira</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>010D - CONGRESO, CÓRDOBA CAPITAL, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>INACTIVO</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>A confirmar por el área</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>4848</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>15625</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>44913</v>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Coincide con la fila 4848 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (15.625 contra 44.913). El tablero conserva la fila 4848 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>4885</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>CÓRDOBA PRODUCTIVA</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Visita a CNH Industrial</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
           <t>TODAS LAS LOCALIDADES</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>PROVINCIA DE CÓRDOBA, ARGENTINA</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Hombres y mujeres desde 26 a 60 años</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>OBSERVADO</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Público afín agricolaganadero, industria, producción</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>INACTIVO</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>A confirmar por el área</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>2818</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Tiene ESTADO = ACTIVO</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>Coincide con la fila 2818 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las métricas son distintas (impresiones 0 en las dos; inversión 207.003 contra 93.405). El tablero conserva la fila 2818 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>A07636</t>
-        </is>
-      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>4881</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>184611</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>53138</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Empate en FECHA DE ENVÍO y ESTADO: se conserva la primera de la planilla</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Coincide con la fila 4881 en campaña, título, plataforma, destino, INICIO, FIN, link, tipo de material y audiencia, pero las impresiones son distintas (184.611 contra 53.138). El tablero conserva la fila 4881 y no suma las métricas. Confirmar si es la misma pieza cargada dos veces o si son piezas distintas; si son distintas, diferenciarlas en la planilla (por ejemplo en el título o el link).</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data(pautas_barrios.json): 6 filas pendientes pasan a entrar, 8.114 entradas — fuente: Pauta RRSS_GLOBAL.xlsx (carga del 23/10)
Mismo crudo que 87a2a14 (sha256 3eebe141f35a6ea8131491aefb9ad6fb8621ab741295cd6e89932b8775b84744),
reglas de a9d9890.
- 979, 1294, 1295 (Obras Julio 2026): pendiente -> toda_capital.
- 1243 (Ampliación Cabildo): pendiente -> circuito_sin_barrio 10M.
- 1529: pendiente -> barrio TEODORO FELS. 1536: pendiente -> barrio VILLA QUISQUIZACATE.
- 23 filas que ya entraban suman la entrada de barrio VILLA QUISQUIZACATE.
- Siguen pendientes 1468 (Pueyrredón, alias sin confirmar) y 1560 (Felipe Varela).
Filas: entran 1.129 (antes 1.123), pendientes 2 (antes 8), duplicadas 34 (sin cambios).
Entradas: 8.114 (antes 8.085): barrios 4.314 en 185 barrios, circuitos_sin_barrio 3.342,
toda_capital 458. Al 23/10 no cambia la pauta activa (210; 108 circuitos, 31 barrios).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Filas_no_procesadas_pauta_capital.xlsx
+++ b/public/data/Filas_no_procesadas_pauta_capital.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duplicadas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$1:$J$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1123</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="6">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8130</v>
+        <v>8159</v>
       </c>
     </row>
     <row r="13">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8085</v>
+        <v>8114</v>
       </c>
     </row>
     <row r="16">
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -790,16 +790,16 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>979</v>
+        <v>1468</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
+          <t>CORDOBESES EN ALERTA</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Obras Julio 2026 (Link)</t>
+          <t>Cordobeses en Alerta Santiago Gomez #51 - B° Pueyrredon (Video)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años</t>
+          <t>Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -824,23 +824,23 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>La localidad es Córdoba Capital pero la AUDIENCIA nombra otro departamento («Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años»). Corregir la localidad o la audiencia.</t>
+          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad)»). Escribir el barrio con su nombre oficial.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>PENDIENTE: la audiencia nombra otro departamento (Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años)</t>
+          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad))</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A05616</t>
+          <t>A06204</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>1243</v>
+        <v>1560</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -849,12 +849,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Puesta en Valor del Centro de Cuidado Infantil y Centro Intregral de Personas Mayores - Ampliación Cabildo</t>
+          <t>Plan 800 Cuadras Felipe Varela</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>010M - AMPLIACION CABILDO, CÓRDOBA CAPITAL, ARGENTINA</t>
+          <t>010C - COMERCIAL, CÓRDOBA CAPITAL, ARGENTINA</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Barrio Ampliación Cabildo de 30 a 60 años sin Advantadge</t>
+          <t>Barrio Felipe Varela de 30 a 60 años sin km agregados</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -874,322 +874,22 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Barrio Ampliación Cabildo de 30 a 60 años sin Advantadge»). Escribir el barrio con su nombre oficial.</t>
+          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Barrio Felipe Varela de 30 a 60 años sin km agregados»). Escribir el barrio con su nombre oficial.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Barrio Ampliación Cabildo de 30 a 60 años sin Advantadge)</t>
+          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Barrio Felipe Varela de 30 a 60 años sin km agregados)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A06014</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>1294</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Obras Julio 2026 (Link)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>CÓRDOBA CAPITAL, DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>La localidad es Córdoba Capital pero la AUDIENCIA nombra otro departamento («Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años»). Corregir la localidad o la audiencia.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra otro departamento (Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años)</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>A05616</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>1295</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Obras Julio 2026 (Link)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>CÓRDOBA CAPITAL, DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>La localidad es Córdoba Capital pero la AUDIENCIA nombra otro departamento («Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años»). Corregir la localidad o la audiencia.</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra otro departamento (Córdoba Capital 30 a 60 años , Departamento Presidente Roque Sáenz Peña 18 a +65 años , Departamento Punilla 18 a +65 años , Departamento San Alberto 18 a +65 años , Departamento Unión 18 a +65 años)</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>A06037</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>1468</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>CORDOBESES EN ALERTA</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Cordobeses en Alerta Santiago Gomez #51 - B° Pueyrredon (Video)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>CÓRDOBA CAPITAL, DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad)»). Escribir el barrio con su nombre oficial.</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Pautar a barrios del cuadrante 8: Pueyrredón y pautar a conjunto de anuncios de Interesados en Seguridad))</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>A06204</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>1529</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Plan Reparación Vial Inegral Av. Duarte Quirós</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>011F - LOS ROBLES, CÓRDOBA CAPITAL, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Barrio Teódoro Fells de 30 a 60 años sin advantage</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Barrio Teódoro Fells de 30 a 60 años sin advantage»). Escribir el barrio con su nombre oficial.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Barrio Teódoro Fells de 30 a 60 años sin advantage)</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>A06283</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>1536</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Obras Avenida Bodereau</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>014C - ARGUELLO SEGUNDO, CÓRDOBA CAPITAL, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Barrio Villa Quizquizacate de 30 a 60 años sin advantage</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Barrio Villa Quizquizacate de 30 a 60 años sin advantage»). Escribir el barrio con su nombre oficial.</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Barrio Villa Quizquizacate de 30 a 60 años sin advantage)</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>A06290</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>1560</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>COMUNICACIÓN INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Plan 800 Cuadras Felipe Varela</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>010C - COMERCIAL, CÓRDOBA CAPITAL, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>DEPARTAMENTO CAPITAL, PROVINCIA DE CÓRDOBA, ARGENTINA</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Barrio Felipe Varela de 30 a 60 años sin km agregados</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>INACTIVO</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>La AUDIENCIA nombra un barrio que no figura con su nombre oficial ni tiene un alias confirmado («Barrio Felipe Varela de 30 a 60 años sin km agregados»). Escribir el barrio con su nombre oficial.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>PENDIENTE: la audiencia nombra un barrio que no se pudo resolver (Barrio Felipe Varela de 30 a 60 años sin km agregados)</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
           <t>A06302</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>